<commit_message>
fix: forgot to deselect intermediate column
</commit_message>
<xml_diff>
--- a/mica/DD_NAKO_P2.R_1.xlsx
+++ b/mica/DD_NAKO_P2.R_1.xlsx
@@ -1713,8 +1713,10 @@
           <t>Mannlich</t>
         </is>
       </c>
-      <c r="E2" t="b">
-        <v>0</v>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
       </c>
     </row>
     <row r="3">
@@ -1736,8 +1738,10 @@
           <t>Weiblich</t>
         </is>
       </c>
-      <c r="E3" t="b">
-        <v>0</v>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
       </c>
     </row>
     <row r="4">
@@ -1759,8 +1763,10 @@
           <t>Missing</t>
         </is>
       </c>
-      <c r="E4" t="b">
-        <v>1</v>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
       </c>
     </row>
     <row r="5">
@@ -1782,8 +1788,10 @@
           <t>Less than primary education (Not applicable for Germany)</t>
         </is>
       </c>
-      <c r="E5" t="b">
-        <v>0</v>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
       </c>
     </row>
     <row r="6">
@@ -1805,8 +1813,10 @@
           <t>Primary education</t>
         </is>
       </c>
-      <c r="E6" t="b">
-        <v>0</v>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
       </c>
     </row>
     <row r="7">
@@ -1828,8 +1838,10 @@
           <t>Lower secondary education</t>
         </is>
       </c>
-      <c r="E7" t="b">
-        <v>0</v>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
       </c>
     </row>
     <row r="8">
@@ -1851,8 +1863,10 @@
           <t>Upper secondary education</t>
         </is>
       </c>
-      <c r="E8" t="b">
-        <v>0</v>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
       </c>
     </row>
     <row r="9">
@@ -1874,8 +1888,10 @@
           <t>Post-secondary non-tertiary education</t>
         </is>
       </c>
-      <c r="E9" t="b">
-        <v>0</v>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
       </c>
     </row>
     <row r="10">
@@ -1897,8 +1913,10 @@
           <t>Short-cycle tertiary education (Not applicable for Germany)</t>
         </is>
       </c>
-      <c r="E10" t="b">
-        <v>0</v>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
       </c>
     </row>
     <row r="11">
@@ -1920,8 +1938,10 @@
           <t>Bachelor's or equivalent level</t>
         </is>
       </c>
-      <c r="E11" t="b">
-        <v>0</v>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
       </c>
     </row>
     <row r="12">
@@ -1943,8 +1963,10 @@
           <t>Master's or equivalent level</t>
         </is>
       </c>
-      <c r="E12" t="b">
-        <v>0</v>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
       </c>
     </row>
     <row r="13">
@@ -1966,8 +1988,10 @@
           <t>Doctoral or equivalent level</t>
         </is>
       </c>
-      <c r="E13" t="b">
-        <v>0</v>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
       </c>
     </row>
     <row r="14">
@@ -1989,8 +2013,10 @@
           <t>Other</t>
         </is>
       </c>
-      <c r="E14" t="b">
-        <v>0</v>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
       </c>
     </row>
     <row r="15">
@@ -2012,8 +2038,10 @@
           <t>Missing</t>
         </is>
       </c>
-      <c r="E15" t="b">
-        <v>1</v>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
       </c>
     </row>
     <row r="16">
@@ -2035,8 +2063,10 @@
           <t>still in general-education school training and without a vocational qualification</t>
         </is>
       </c>
-      <c r="E16" t="b">
-        <v>1</v>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
       </c>
     </row>
     <row r="17">
@@ -2058,8 +2088,10 @@
           <t>still in vocational training</t>
         </is>
       </c>
-      <c r="E17" t="b">
-        <v>1</v>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
       </c>
     </row>
     <row r="18">
@@ -2081,8 +2113,10 @@
           <t>Missing</t>
         </is>
       </c>
-      <c r="E18" t="b">
-        <v>1</v>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
       </c>
     </row>
     <row r="19">
@@ -2104,8 +2138,10 @@
           <t>Kein Raucher, auch nicht ehemalig</t>
         </is>
       </c>
-      <c r="E19" t="b">
-        <v>0</v>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
       </c>
     </row>
     <row r="20">
@@ -2127,8 +2163,10 @@
           <t>Ehemaliger Raucher</t>
         </is>
       </c>
-      <c r="E20" t="b">
-        <v>0</v>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
       </c>
     </row>
     <row r="21">
@@ -2150,8 +2188,10 @@
           <t>Raucher</t>
         </is>
       </c>
-      <c r="E21" t="b">
-        <v>0</v>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
       </c>
     </row>
     <row r="22">
@@ -2173,8 +2213,10 @@
           <t>Rauchstatus unbekannt</t>
         </is>
       </c>
-      <c r="E22" t="b">
-        <v>0</v>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
       </c>
     </row>
     <row r="23">
@@ -2196,8 +2238,10 @@
           <t>missing due to impossible calculation</t>
         </is>
       </c>
-      <c r="E23" t="b">
-        <v>1</v>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
       </c>
     </row>
     <row r="24">
@@ -2219,8 +2263,10 @@
           <t>Implausible information</t>
         </is>
       </c>
-      <c r="E24" t="b">
-        <v>1</v>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
       </c>
     </row>
     <row r="25">
@@ -2242,8 +2288,10 @@
           <t>Calculation not possible due to implausible values</t>
         </is>
       </c>
-      <c r="E25" t="b">
-        <v>1</v>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
       </c>
     </row>
     <row r="26">
@@ -2265,8 +2313,10 @@
           <t>Allowed skipped</t>
         </is>
       </c>
-      <c r="E26" t="b">
-        <v>1</v>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
       </c>
     </row>
     <row r="27">
@@ -2288,8 +2338,10 @@
           <t>Not specified</t>
         </is>
       </c>
-      <c r="E27" t="b">
-        <v>1</v>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
       </c>
     </row>
     <row r="28">
@@ -2311,8 +2363,10 @@
           <t>Don't know</t>
         </is>
       </c>
-      <c r="E28" t="b">
-        <v>1</v>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
       </c>
     </row>
     <row r="29">
@@ -2334,8 +2388,10 @@
           <t>Not specified, erroneously skipped</t>
         </is>
       </c>
-      <c r="E29" t="b">
-        <v>1</v>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
       </c>
     </row>
     <row r="30">
@@ -2357,8 +2413,10 @@
           <t>I don't know</t>
         </is>
       </c>
-      <c r="E30" t="b">
-        <v>1</v>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
       </c>
     </row>
     <row r="31">
@@ -2380,8 +2438,10 @@
           <t>no answer</t>
         </is>
       </c>
-      <c r="E31" t="b">
-        <v>1</v>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
       </c>
     </row>
     <row r="32">
@@ -2403,8 +2463,10 @@
           <t>implausible</t>
         </is>
       </c>
-      <c r="E32" t="b">
-        <v>1</v>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
       </c>
     </row>
     <row r="33">
@@ -2426,8 +2488,10 @@
           <t>Ja</t>
         </is>
       </c>
-      <c r="E33" t="b">
-        <v>0</v>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
       </c>
     </row>
     <row r="34">
@@ -2449,8 +2513,10 @@
           <t>Nein</t>
         </is>
       </c>
-      <c r="E34" t="b">
-        <v>0</v>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
       </c>
     </row>
     <row r="35">
@@ -2472,8 +2538,10 @@
           <t>I don't know</t>
         </is>
       </c>
-      <c r="E35" t="b">
-        <v>1</v>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
       </c>
     </row>
     <row r="36">
@@ -2495,8 +2563,10 @@
           <t>no answer</t>
         </is>
       </c>
-      <c r="E36" t="b">
-        <v>1</v>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
       </c>
     </row>
     <row r="37">
@@ -2518,8 +2588,10 @@
           <t>Ja</t>
         </is>
       </c>
-      <c r="E37" t="b">
-        <v>0</v>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
       </c>
     </row>
     <row r="38">
@@ -2541,8 +2613,10 @@
           <t>Nein</t>
         </is>
       </c>
-      <c r="E38" t="b">
-        <v>0</v>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
       </c>
     </row>
     <row r="39">
@@ -2564,8 +2638,10 @@
           <t>I don't know</t>
         </is>
       </c>
-      <c r="E39" t="b">
-        <v>1</v>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
       </c>
     </row>
     <row r="40">
@@ -2587,8 +2663,10 @@
           <t>no answer</t>
         </is>
       </c>
-      <c r="E40" t="b">
-        <v>1</v>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
       </c>
     </row>
     <row r="41">
@@ -2610,8 +2688,10 @@
           <t>Ja</t>
         </is>
       </c>
-      <c r="E41" t="b">
-        <v>0</v>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
       </c>
     </row>
     <row r="42">
@@ -2633,8 +2713,10 @@
           <t>Nein</t>
         </is>
       </c>
-      <c r="E42" t="b">
-        <v>0</v>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
       </c>
     </row>
     <row r="43">
@@ -2656,8 +2738,10 @@
           <t>missing</t>
         </is>
       </c>
-      <c r="E43" t="b">
-        <v>1</v>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
       </c>
     </row>
     <row r="44">
@@ -2679,8 +2763,10 @@
           <t>Ja</t>
         </is>
       </c>
-      <c r="E44" t="b">
-        <v>0</v>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
       </c>
     </row>
     <row r="45">
@@ -2702,8 +2788,10 @@
           <t>Nein</t>
         </is>
       </c>
-      <c r="E45" t="b">
-        <v>0</v>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
       </c>
     </row>
     <row r="46">
@@ -2725,8 +2813,10 @@
           <t>I don't know</t>
         </is>
       </c>
-      <c r="E46" t="b">
-        <v>1</v>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
       </c>
     </row>
     <row r="47">
@@ -2748,8 +2838,10 @@
           <t>no answer</t>
         </is>
       </c>
-      <c r="E47" t="b">
-        <v>1</v>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
       </c>
     </row>
     <row r="48">
@@ -2771,8 +2863,10 @@
           <t>Sample too old</t>
         </is>
       </c>
-      <c r="E48" t="b">
-        <v>1</v>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
       </c>
     </row>
     <row r="49">
@@ -2794,8 +2888,10 @@
           <t>Hemolytic sample</t>
         </is>
       </c>
-      <c r="E49" t="b">
-        <v>1</v>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
       </c>
     </row>
     <row r="50">
@@ -2817,8 +2913,10 @@
           <t>lipemic sample</t>
         </is>
       </c>
-      <c r="E50" t="b">
-        <v>1</v>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
       </c>
     </row>
     <row r="51">
@@ -2840,8 +2938,10 @@
           <t>Technically not possible</t>
         </is>
       </c>
-      <c r="E51" t="b">
-        <v>1</v>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
       </c>
     </row>
     <row r="52">
@@ -2863,8 +2963,10 @@
           <t>Planned not determined</t>
         </is>
       </c>
-      <c r="E52" t="b">
-        <v>1</v>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
       </c>
     </row>
     <row r="53">
@@ -2886,8 +2988,10 @@
           <t>no valid information available</t>
         </is>
       </c>
-      <c r="E53" t="b">
-        <v>1</v>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
       </c>
     </row>
     <row r="54">
@@ -2909,8 +3013,10 @@
           <t>Sample too old</t>
         </is>
       </c>
-      <c r="E54" t="b">
-        <v>1</v>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
       </c>
     </row>
     <row r="55">
@@ -2932,8 +3038,10 @@
           <t>Hemolytic sample</t>
         </is>
       </c>
-      <c r="E55" t="b">
-        <v>1</v>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
       </c>
     </row>
     <row r="56">
@@ -2955,8 +3063,10 @@
           <t>lipemic sample</t>
         </is>
       </c>
-      <c r="E56" t="b">
-        <v>1</v>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
       </c>
     </row>
     <row r="57">
@@ -2978,8 +3088,10 @@
           <t>Technically not possible</t>
         </is>
       </c>
-      <c r="E57" t="b">
-        <v>1</v>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
       </c>
     </row>
     <row r="58">
@@ -3001,8 +3113,10 @@
           <t>Planned not determined</t>
         </is>
       </c>
-      <c r="E58" t="b">
-        <v>1</v>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
       </c>
     </row>
     <row r="59">
@@ -3024,8 +3138,10 @@
           <t>no valid information available</t>
         </is>
       </c>
-      <c r="E59" t="b">
-        <v>1</v>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
       </c>
     </row>
     <row r="60">
@@ -3047,8 +3163,10 @@
           <t>Eliminated by group of experts</t>
         </is>
       </c>
-      <c r="E60" t="b">
-        <v>1</v>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
       </c>
     </row>
     <row r="61">
@@ -3070,8 +3188,10 @@
           <t>Sample too old</t>
         </is>
       </c>
-      <c r="E61" t="b">
-        <v>1</v>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
       </c>
     </row>
     <row r="62">
@@ -3093,8 +3213,10 @@
           <t>Hemolytic sample</t>
         </is>
       </c>
-      <c r="E62" t="b">
-        <v>1</v>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
       </c>
     </row>
     <row r="63">
@@ -3116,8 +3238,10 @@
           <t>lipemic sample</t>
         </is>
       </c>
-      <c r="E63" t="b">
-        <v>1</v>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
       </c>
     </row>
     <row r="64">
@@ -3139,8 +3263,10 @@
           <t>Technically not possible</t>
         </is>
       </c>
-      <c r="E64" t="b">
-        <v>1</v>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
       </c>
     </row>
     <row r="65">
@@ -3162,8 +3288,10 @@
           <t>Planned not determined</t>
         </is>
       </c>
-      <c r="E65" t="b">
-        <v>1</v>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
       </c>
     </row>
     <row r="66">
@@ -3185,8 +3313,10 @@
           <t>no valid information available</t>
         </is>
       </c>
-      <c r="E66" t="b">
-        <v>1</v>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
       </c>
     </row>
     <row r="67">
@@ -3208,8 +3338,10 @@
           <t>Eliminated by group of experts</t>
         </is>
       </c>
-      <c r="E67" t="b">
-        <v>1</v>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
       </c>
     </row>
     <row r="68">
@@ -3231,8 +3363,10 @@
           <t>missing due to impossible calculation</t>
         </is>
       </c>
-      <c r="E68" t="b">
-        <v>1</v>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
       </c>
     </row>
     <row r="69">
@@ -3254,8 +3388,10 @@
           <t>Implausible information</t>
         </is>
       </c>
-      <c r="E69" t="b">
-        <v>1</v>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
       </c>
     </row>
     <row r="70">
@@ -3277,8 +3413,10 @@
           <t>Calculation not possible due to implausible values</t>
         </is>
       </c>
-      <c r="E70" t="b">
-        <v>1</v>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
       </c>
     </row>
     <row r="71">
@@ -3300,8 +3438,10 @@
           <t>Allowed skipped</t>
         </is>
       </c>
-      <c r="E71" t="b">
-        <v>1</v>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
       </c>
     </row>
     <row r="72">
@@ -3323,8 +3463,10 @@
           <t>Not specified</t>
         </is>
       </c>
-      <c r="E72" t="b">
-        <v>1</v>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
       </c>
     </row>
     <row r="73">
@@ -3346,8 +3488,10 @@
           <t>Don't know</t>
         </is>
       </c>
-      <c r="E73" t="b">
-        <v>1</v>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
       </c>
     </row>
     <row r="74">
@@ -3369,8 +3513,10 @@
           <t>Not specified, erroneously skipped</t>
         </is>
       </c>
-      <c r="E74" t="b">
-        <v>1</v>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
       </c>
     </row>
     <row r="75">
@@ -3392,8 +3538,10 @@
           <t>missing data</t>
         </is>
       </c>
-      <c r="E75" t="b">
-        <v>1</v>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
       </c>
     </row>
     <row r="76">
@@ -3415,8 +3563,10 @@
           <t>Implausible information</t>
         </is>
       </c>
-      <c r="E76" t="b">
-        <v>1</v>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
       </c>
     </row>
     <row r="77">
@@ -3438,8 +3588,10 @@
           <t>calculation not possible due to implausible</t>
         </is>
       </c>
-      <c r="E77" t="b">
-        <v>1</v>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
       </c>
     </row>
     <row r="78">
@@ -3461,8 +3613,10 @@
           <t>Allowed skipped</t>
         </is>
       </c>
-      <c r="E78" t="b">
-        <v>1</v>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
       </c>
     </row>
     <row r="79">
@@ -3484,8 +3638,10 @@
           <t>Not specified</t>
         </is>
       </c>
-      <c r="E79" t="b">
-        <v>1</v>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
       </c>
     </row>
     <row r="80">
@@ -3507,8 +3663,10 @@
           <t>Don't know</t>
         </is>
       </c>
-      <c r="E80" t="b">
-        <v>1</v>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
       </c>
     </row>
     <row r="81">
@@ -3530,8 +3688,10 @@
           <t>Not specified, erroneously skipped</t>
         </is>
       </c>
-      <c r="E81" t="b">
-        <v>1</v>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
       </c>
     </row>
     <row r="82">
@@ -3553,8 +3713,10 @@
           <t>missing</t>
         </is>
       </c>
-      <c r="E82" t="b">
-        <v>1</v>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
       </c>
     </row>
     <row r="83">
@@ -3576,8 +3738,10 @@
           <t>missing</t>
         </is>
       </c>
-      <c r="E83" t="b">
-        <v>1</v>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
       </c>
     </row>
     <row r="84">
@@ -3599,8 +3763,10 @@
           <t>missing</t>
         </is>
       </c>
-      <c r="E84" t="b">
-        <v>1</v>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
       </c>
     </row>
     <row r="85">
@@ -3622,8 +3788,10 @@
           <t>missing</t>
         </is>
       </c>
-      <c r="E85" t="b">
-        <v>1</v>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>